<commit_message>
occ change by education and training
</commit_message>
<xml_diff>
--- a/data/processed/sam_auto_dashboard_2024_refresh/occ_change_by_education/segment_occ_change_by_education_2024_2030.xlsx
+++ b/data/processed/sam_auto_dashboard_2024_refresh/occ_change_by_education/segment_occ_change_by_education_2024_2030.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="34">
   <si>
     <t>methodology</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>pct_change</t>
+  </si>
+  <si>
+    <t>share_base</t>
+  </si>
+  <si>
+    <t>share_target</t>
+  </si>
+  <si>
+    <t>share_change</t>
   </si>
   <si>
     <t>sam_mi_moodys_mi</t>
@@ -90,16 +99,16 @@
     <t>BA+</t>
   </si>
   <si>
+    <t>SC or Associate's</t>
+  </si>
+  <si>
     <t>HS or Less</t>
   </si>
   <si>
-    <t>SC or Associate's</t>
+    <t>SC/Associate or Employer Training</t>
   </si>
   <si>
     <t>HS or Less - Limited Training</t>
-  </si>
-  <si>
-    <t>SC/Associate or Employer Training</t>
   </si>
   <si>
     <t>Associate's</t>
@@ -466,10 +475,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -500,25 +509,34 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G2">
         <v>3451.96904055808</v>
@@ -532,89 +550,116 @@
       <c r="J2">
         <v>-0.04342635557299448</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2">
+        <v>0.1624634248293149</v>
+      </c>
+      <c r="L2">
+        <v>0.1680227242756014</v>
+      </c>
+      <c r="M2">
+        <v>0.09397388447319011</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G3">
-        <v>16795.04319647182</v>
+        <v>1000.656548635188</v>
       </c>
       <c r="H3">
-        <v>15430.95372287424</v>
+        <v>919.4599649326431</v>
       </c>
       <c r="I3">
-        <v>-1364.089473597583</v>
+        <v>-81.19658370254444</v>
       </c>
       <c r="J3">
-        <v>-0.08121976571540711</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>-0.08114330917365188</v>
+      </c>
+      <c r="K3">
+        <v>0.04709488644280301</v>
+      </c>
+      <c r="L3">
+        <v>0.04678595975420354</v>
+      </c>
+      <c r="M3">
+        <v>0.05090080607536579</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G4">
-        <v>1000.656548635188</v>
+        <v>16795.04319647182</v>
       </c>
       <c r="H4">
-        <v>919.4599649326431</v>
+        <v>15430.95372287424</v>
       </c>
       <c r="I4">
-        <v>-81.19658370254444</v>
+        <v>-1364.089473597583</v>
       </c>
       <c r="J4">
-        <v>-0.08114330917365188</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>-0.08121976571540711</v>
+      </c>
+      <c r="K4">
+        <v>0.7904416887278821</v>
+      </c>
+      <c r="L4">
+        <v>0.7851913159701951</v>
+      </c>
+      <c r="M4">
+        <v>0.855125309451444</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D5">
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G5">
         <v>1664.428681321303</v>
@@ -628,89 +673,116 @@
       <c r="J5">
         <v>0.00756879904398951</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5">
+        <v>0.2665394402035619</v>
+      </c>
+      <c r="L5">
+        <v>0.2745862662578333</v>
+      </c>
+      <c r="M5">
+        <v>-0.0918734664611702</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>3887.639306570689</v>
+        <v>692.5188546786338</v>
       </c>
       <c r="H6">
-        <v>3774.373398713734</v>
+        <v>656.0666391380176</v>
       </c>
       <c r="I6">
-        <v>-113.2659078569554</v>
+        <v>-36.45221554061618</v>
       </c>
       <c r="J6">
-        <v>-0.02913488081713733</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>-0.05263714524788207</v>
+      </c>
+      <c r="K6">
+        <v>0.1108990670059372</v>
+      </c>
+      <c r="L6">
+        <v>0.1074204246564072</v>
+      </c>
+      <c r="M6">
+        <v>0.2658409418933974</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G7">
-        <v>692.5188546786338</v>
+        <v>3887.639306570689</v>
       </c>
       <c r="H7">
-        <v>656.0666391380176</v>
+        <v>3774.373398713734</v>
       </c>
       <c r="I7">
-        <v>-36.45221554061618</v>
+        <v>-113.2659078569554</v>
       </c>
       <c r="J7">
-        <v>-0.05263714524788207</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>-0.02913488081713733</v>
+      </c>
+      <c r="K7">
+        <v>0.6225614927905009</v>
+      </c>
+      <c r="L7">
+        <v>0.6179933090857594</v>
+      </c>
+      <c r="M7">
+        <v>0.8260325245677729</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G8">
         <v>1144.895853088782</v>
@@ -724,89 +796,116 @@
       <c r="J8">
         <v>-0.1333446500349006</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8">
+        <v>0.1268844221105523</v>
+      </c>
+      <c r="L8">
+        <v>0.1328344022444252</v>
+      </c>
+      <c r="M8">
+        <v>0.09827450286914931</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D9">
         <v>3</v>
       </c>
       <c r="E9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G9">
-        <v>7470.162051341688</v>
+        <v>408.0816902098634</v>
       </c>
       <c r="H9">
-        <v>6145.380291756315</v>
+        <v>332.0668703905082</v>
       </c>
       <c r="I9">
-        <v>-1324.781759585373</v>
+        <v>-76.01481981935524</v>
       </c>
       <c r="J9">
-        <v>-0.1773431085537741</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>-0.1862735369976125</v>
+      </c>
+      <c r="K9">
+        <v>0.04522613065326623</v>
+      </c>
+      <c r="L9">
+        <v>0.04445531687850469</v>
+      </c>
+      <c r="M9">
+        <v>0.04893251611168861</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <v>3</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G10">
-        <v>408.0816902098634</v>
+        <v>7470.162051341688</v>
       </c>
       <c r="H10">
-        <v>332.0668703905082</v>
+        <v>6145.380291756315</v>
       </c>
       <c r="I10">
-        <v>-76.01481981935524</v>
+        <v>-1324.781759585373</v>
       </c>
       <c r="J10">
-        <v>-0.1862735369976125</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>-0.1773431085537741</v>
+      </c>
+      <c r="K10">
+        <v>0.8278894472361815</v>
+      </c>
+      <c r="L10">
+        <v>0.8227102808770701</v>
+      </c>
+      <c r="M10">
+        <v>0.8527929810191622</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D11">
         <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G11">
         <v>2548.713461124355</v>
@@ -820,89 +919,116 @@
       <c r="J11">
         <v>-0.00222421536994241</v>
       </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="K11">
+        <v>0.1706372264187481</v>
+      </c>
+      <c r="L11">
+        <v>0.1789737600560029</v>
+      </c>
+      <c r="M11">
+        <v>0.00779326410643654</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D12">
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G12">
-        <v>11600.84106595768</v>
+        <v>786.889967566202</v>
       </c>
       <c r="H12">
-        <v>10915.53795803819</v>
+        <v>750.4533219861942</v>
       </c>
       <c r="I12">
-        <v>-685.3031079194952</v>
+        <v>-36.43664558000785</v>
       </c>
       <c r="J12">
-        <v>-0.05907357096120355</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>-0.0463046259093936</v>
+      </c>
+      <c r="K12">
+        <v>0.05268254890567475</v>
+      </c>
+      <c r="L12">
+        <v>0.05281521770540181</v>
+      </c>
+      <c r="M12">
+        <v>0.05009102658202839</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D13">
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G13">
-        <v>786.889967566202</v>
+        <v>11600.84106595768</v>
       </c>
       <c r="H13">
-        <v>750.4533219861942</v>
+        <v>10915.53795803819</v>
       </c>
       <c r="I13">
-        <v>-36.43664558000785</v>
+        <v>-685.3031079194952</v>
       </c>
       <c r="J13">
-        <v>-0.0463046259093936</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
+        <v>-0.05907357096120355</v>
+      </c>
+      <c r="K13">
+        <v>0.7766802246755772</v>
+      </c>
+      <c r="L13">
+        <v>0.7682110222385953</v>
+      </c>
+      <c r="M13">
+        <v>0.9421157093115351</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G14">
         <v>2443.987754662811</v>
@@ -916,89 +1042,116 @@
       <c r="J14">
         <v>-0.01431517488000416</v>
       </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="K14">
+        <v>0.4082140634723086</v>
+      </c>
+      <c r="L14">
+        <v>0.4104836703607108</v>
+      </c>
+      <c r="M14">
+        <v>0.2956548262474077</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D15">
         <v>5</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F15" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G15">
-        <v>3200.282745816092</v>
+        <v>342.7543802271001</v>
       </c>
       <c r="H15">
-        <v>3140.045112583321</v>
+        <v>319.6438079607781</v>
       </c>
       <c r="I15">
-        <v>-60.23763323277126</v>
+        <v>-23.11057226632204</v>
       </c>
       <c r="J15">
-        <v>-0.01882259725692153</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+        <v>-0.06742604500344992</v>
+      </c>
+      <c r="K15">
+        <v>0.05724953329184791</v>
+      </c>
+      <c r="L15">
+        <v>0.05446595020205714</v>
+      </c>
+      <c r="M15">
+        <v>0.1952989862345808</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D16">
         <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G16">
-        <v>342.7543802271001</v>
+        <v>3200.282745816092</v>
       </c>
       <c r="H16">
-        <v>319.6438079607781</v>
+        <v>3140.045112583321</v>
       </c>
       <c r="I16">
-        <v>-23.11057226632204</v>
+        <v>-60.23763323277126</v>
       </c>
       <c r="J16">
-        <v>-0.06742604500344992</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>-0.01882259725692153</v>
+      </c>
+      <c r="K16">
+        <v>0.5345364032358435</v>
+      </c>
+      <c r="L16">
+        <v>0.5350503794372321</v>
+      </c>
+      <c r="M16">
+        <v>0.5090461875180115</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D17">
         <v>6</v>
       </c>
       <c r="E17" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G17">
         <v>737.9275791029602</v>
@@ -1012,89 +1165,116 @@
       <c r="J17">
         <v>0.02527738081884549</v>
       </c>
-    </row>
-    <row r="18" spans="1:10">
+      <c r="K17">
+        <v>0.7150284321689701</v>
+      </c>
+      <c r="L17">
+        <v>0.7220370319238563</v>
+      </c>
+      <c r="M17">
+        <v>1.179358721779987</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D18">
         <v>6</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F18" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G18">
-        <v>199.9497019041748</v>
+        <v>94.14822441861125</v>
       </c>
       <c r="H18">
-        <v>197.2497972978348</v>
+        <v>94.01137035866383</v>
       </c>
       <c r="I18">
-        <v>-2.699904606339999</v>
+        <v>-0.1368540599474244</v>
       </c>
       <c r="J18">
-        <v>-0.01350291888724055</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
+        <v>-0.00145360213421477</v>
+      </c>
+      <c r="K18">
+        <v>0.09122664500406108</v>
+      </c>
+      <c r="L18">
+        <v>0.08971906467331897</v>
+      </c>
+      <c r="M18">
+        <v>-0.008652822516867839</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D19">
         <v>6</v>
       </c>
       <c r="E19" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F19" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G19">
-        <v>94.14822441861125</v>
+        <v>199.9497019041748</v>
       </c>
       <c r="H19">
-        <v>94.01137035866383</v>
+        <v>197.2497972978348</v>
       </c>
       <c r="I19">
-        <v>-0.1368540599474244</v>
+        <v>-2.699904606339999</v>
       </c>
       <c r="J19">
-        <v>-0.00145360213421477</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
+        <v>-0.01350291888724055</v>
+      </c>
+      <c r="K19">
+        <v>0.1937449228269689</v>
+      </c>
+      <c r="L19">
+        <v>0.1882439034028248</v>
+      </c>
+      <c r="M19">
+        <v>-0.1707058992631195</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D20">
         <v>7</v>
       </c>
       <c r="E20" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F20" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G20">
         <v>28420.73848797222</v>
@@ -1108,89 +1288,116 @@
       <c r="J20">
         <v>0.03719956910429145</v>
       </c>
-    </row>
-    <row r="21" spans="1:10">
+      <c r="K20">
+        <v>0.1642038946162641</v>
+      </c>
+      <c r="L20">
+        <v>0.1684715681373224</v>
+      </c>
+      <c r="M20">
+        <v>0.5590864708306096</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D21">
         <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F21" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G21">
-        <v>136344.2054982822</v>
+        <v>8317.056013745616</v>
       </c>
       <c r="H21">
-        <v>137595.4236138235</v>
+        <v>7899.610672826003</v>
       </c>
       <c r="I21">
-        <v>1251.218115541269</v>
+        <v>-417.445340919613</v>
       </c>
       <c r="J21">
-        <v>0.009176907159116735</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
+        <v>-0.05019147883935136</v>
+      </c>
+      <c r="K21">
+        <v>0.04805269186712435</v>
+      </c>
+      <c r="L21">
+        <v>0.04514759494924853</v>
+      </c>
+      <c r="M21">
+        <v>-0.2207523489642682</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D22">
         <v>7</v>
       </c>
       <c r="E22" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F22" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G22">
-        <v>8317.056013745616</v>
+        <v>136344.2054982822</v>
       </c>
       <c r="H22">
-        <v>7899.610672826003</v>
+        <v>137595.4236138235</v>
       </c>
       <c r="I22">
-        <v>-417.445340919613</v>
+        <v>1251.218115541269</v>
       </c>
       <c r="J22">
-        <v>-0.05019147883935136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
+        <v>0.009176907159116735</v>
+      </c>
+      <c r="K22">
+        <v>0.7877434135166117</v>
+      </c>
+      <c r="L22">
+        <v>0.7863808369134291</v>
+      </c>
+      <c r="M22">
+        <v>0.6616658781336586</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D23">
         <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F23" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G23">
         <v>19646.96893063571</v>
@@ -1204,89 +1411,116 @@
       <c r="J23">
         <v>0.05442807630137755</v>
       </c>
-    </row>
-    <row r="24" spans="1:10">
+      <c r="K23">
+        <v>0.1703395953757215</v>
+      </c>
+      <c r="L23">
+        <v>0.1771289185151771</v>
+      </c>
+      <c r="M23">
+        <v>0.6616646788393189</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F24" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G24">
-        <v>87775.90679190768</v>
+        <v>7917.124277456613</v>
       </c>
       <c r="H24">
-        <v>88145.03513062403</v>
+        <v>8094.795214692798</v>
       </c>
       <c r="I24">
-        <v>369.1283387163567</v>
+        <v>177.6709372361856</v>
       </c>
       <c r="J24">
-        <v>0.004205349192136032</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
+        <v>0.02244134751580061</v>
+      </c>
+      <c r="K24">
+        <v>0.06864161849710952</v>
+      </c>
+      <c r="L24">
+        <v>0.06921222604832412</v>
+      </c>
+      <c r="M24">
+        <v>0.1099349546613908</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D25">
         <v>8</v>
       </c>
       <c r="E25" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F25" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G25">
-        <v>7917.124277456613</v>
+        <v>87775.90679190768</v>
       </c>
       <c r="H25">
-        <v>8094.795214692798</v>
+        <v>88145.03513062403</v>
       </c>
       <c r="I25">
-        <v>177.6709372361856</v>
+        <v>369.1283387163567</v>
       </c>
       <c r="J25">
-        <v>0.02244134751580061</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10">
+        <v>0.004205349192136032</v>
+      </c>
+      <c r="K25">
+        <v>0.761018786127169</v>
+      </c>
+      <c r="L25">
+        <v>0.7536588554364988</v>
+      </c>
+      <c r="M25">
+        <v>0.2284003664992902</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D26">
         <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F26" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G26">
         <v>6147.44206383908</v>
@@ -1300,89 +1534,116 @@
       <c r="J26">
         <v>0.02481979087750858</v>
       </c>
-    </row>
-    <row r="27" spans="1:10">
+      <c r="K26">
+        <v>0.08832531700918218</v>
+      </c>
+      <c r="L26">
+        <v>0.08787128903718494</v>
+      </c>
+      <c r="M26">
+        <v>0.0727948164488649</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D27">
         <v>9</v>
       </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G27">
-        <v>45578.31219938782</v>
+        <v>17874.24573677311</v>
       </c>
       <c r="H27">
-        <v>46745.44486404282</v>
+        <v>18650.53884566201</v>
       </c>
       <c r="I27">
-        <v>1167.132664655001</v>
+        <v>776.2931088889018</v>
       </c>
       <c r="J27">
-        <v>0.02560719360447658</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10">
+        <v>0.04343081774308472</v>
+      </c>
+      <c r="K27">
+        <v>0.2568138755283492</v>
+      </c>
+      <c r="L27">
+        <v>0.2601335891141439</v>
+      </c>
+      <c r="M27">
+        <v>0.3703681428513048</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D28">
         <v>9</v>
       </c>
       <c r="E28" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F28" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G28">
-        <v>17874.24573677311</v>
+        <v>45578.31219938782</v>
       </c>
       <c r="H28">
-        <v>18650.53884566201</v>
+        <v>46745.44486404282</v>
       </c>
       <c r="I28">
-        <v>776.2931088889018</v>
+        <v>1167.132664655001</v>
       </c>
       <c r="J28">
-        <v>0.04343081774308472</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10">
+        <v>0.02560719360447658</v>
+      </c>
+      <c r="K28">
+        <v>0.6548608074624687</v>
+      </c>
+      <c r="L28">
+        <v>0.6519951218486713</v>
+      </c>
+      <c r="M28">
+        <v>0.5568370406998303</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D29">
         <v>10</v>
       </c>
       <c r="E29" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F29" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G29">
         <v>3914.073253833027</v>
@@ -1396,69 +1657,96 @@
       <c r="J29">
         <v>-0.07983986820489161</v>
       </c>
-    </row>
-    <row r="30" spans="1:10">
+      <c r="K29">
+        <v>0.08347529812606426</v>
+      </c>
+      <c r="L29">
+        <v>0.08631932144470537</v>
+      </c>
+      <c r="M29">
+        <v>0.06050142033165728</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D30">
         <v>10</v>
       </c>
       <c r="E30" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F30" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G30">
-        <v>15786.09646507664</v>
+        <v>27188.83028109034</v>
       </c>
       <c r="H30">
-        <v>13984.24805922004</v>
+        <v>24138.02477967726</v>
       </c>
       <c r="I30">
-        <v>-1801.848405856592</v>
+        <v>-3050.80550141308</v>
       </c>
       <c r="J30">
-        <v>-0.1141414794875222</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
+        <v>-0.1122080453580563</v>
+      </c>
+      <c r="K30">
+        <v>0.5798551959114151</v>
+      </c>
+      <c r="L30">
+        <v>0.5785186773328274</v>
+      </c>
+      <c r="M30">
+        <v>0.5906515259883075</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D31">
         <v>10</v>
       </c>
       <c r="E31" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F31" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G31">
-        <v>27188.83028109034</v>
+        <v>15786.09646507664</v>
       </c>
       <c r="H31">
-        <v>24138.02477967726</v>
+        <v>13984.24805922004</v>
       </c>
       <c r="I31">
-        <v>-3050.80550141308</v>
+        <v>-1801.848405856592</v>
       </c>
       <c r="J31">
-        <v>-0.1122080453580563</v>
+        <v>-0.1141414794875222</v>
+      </c>
+      <c r="K31">
+        <v>0.3366695059625208</v>
+      </c>
+      <c r="L31">
+        <v>0.3351620012224674</v>
+      </c>
+      <c r="M31">
+        <v>0.3488470536800351</v>
       </c>
     </row>
   </sheetData>
@@ -1468,10 +1756,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1502,25 +1790,34 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G2">
         <v>3451.96904055808</v>
@@ -1534,89 +1831,116 @@
       <c r="J2">
         <v>-0.04342635557299448</v>
       </c>
-    </row>
-    <row r="3" spans="1:10">
+      <c r="K2">
+        <v>0.1624634248293149</v>
+      </c>
+      <c r="L2">
+        <v>0.1680227242756013</v>
+      </c>
+      <c r="M2">
+        <v>0.09397388447319019</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G3">
-        <v>4414.138798861176</v>
+        <v>13381.56094624583</v>
       </c>
       <c r="H3">
-        <v>4047.357726494847</v>
+        <v>12303.05596131204</v>
       </c>
       <c r="I3">
-        <v>-366.7810723663292</v>
+        <v>-1078.504984933797</v>
       </c>
       <c r="J3">
-        <v>-0.08309232878244716</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>-0.08059635114813489</v>
+      </c>
+      <c r="K3">
+        <v>0.6297896056848274</v>
+      </c>
+      <c r="L3">
+        <v>0.6260308257160782</v>
+      </c>
+      <c r="M3">
+        <v>0.6760970792877125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G4">
-        <v>13381.56094624583</v>
+        <v>4414.138798861176</v>
       </c>
       <c r="H4">
-        <v>12303.05596131204</v>
+        <v>4047.357726494847</v>
       </c>
       <c r="I4">
-        <v>-1078.504984933797</v>
+        <v>-366.7810723663292</v>
       </c>
       <c r="J4">
-        <v>-0.08059635114813489</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>-0.08309232878244716</v>
+      </c>
+      <c r="K4">
+        <v>0.2077469694858577</v>
+      </c>
+      <c r="L4">
+        <v>0.2059464500083204</v>
+      </c>
+      <c r="M4">
+        <v>0.2299290362390974</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D5">
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G5">
         <v>1664.428681321303</v>
@@ -1630,89 +1954,116 @@
       <c r="J5">
         <v>0.00756879904398951</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5">
+        <v>0.2665394402035619</v>
+      </c>
+      <c r="L5">
+        <v>0.2745862662578333</v>
+      </c>
+      <c r="M5">
+        <v>-0.09187346646117028</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G6">
-        <v>855.3865776718878</v>
+        <v>3724.771583577435</v>
       </c>
       <c r="H6">
-        <v>824.1859100788801</v>
+        <v>3606.254127772871</v>
       </c>
       <c r="I6">
-        <v>-31.20066759300778</v>
+        <v>-118.5174558045637</v>
       </c>
       <c r="J6">
-        <v>-0.03647551692700963</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>-0.031818717777785</v>
+      </c>
+      <c r="K6">
+        <v>0.5964800678541141</v>
+      </c>
+      <c r="L6">
+        <v>0.5904664659267769</v>
+      </c>
+      <c r="M6">
+        <v>0.864331333901735</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G7">
-        <v>3724.771583577435</v>
+        <v>855.3865776718878</v>
       </c>
       <c r="H7">
-        <v>3606.254127772871</v>
+        <v>824.1859100788801</v>
       </c>
       <c r="I7">
-        <v>-118.5174558045637</v>
+        <v>-31.20066759300778</v>
       </c>
       <c r="J7">
-        <v>-0.031818717777785</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>-0.03647551692700963</v>
+      </c>
+      <c r="K7">
+        <v>0.136980491942324</v>
+      </c>
+      <c r="L7">
+        <v>0.1349472678153898</v>
+      </c>
+      <c r="M7">
+        <v>0.2275421325594353</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D8">
         <v>3</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G8">
         <v>1144.895853088782</v>
@@ -1726,89 +2077,116 @@
       <c r="J8">
         <v>-0.1333446500349006</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8">
+        <v>0.1268844221105523</v>
+      </c>
+      <c r="L8">
+        <v>0.1328344022444252</v>
+      </c>
+      <c r="M8">
+        <v>0.09827450286914925</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D9">
         <v>3</v>
       </c>
       <c r="E9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G9">
-        <v>1592.652152069054</v>
+        <v>6285.591589482498</v>
       </c>
       <c r="H9">
-        <v>1329.866189055798</v>
+        <v>5147.580973091025</v>
       </c>
       <c r="I9">
-        <v>-262.7859630132555</v>
+        <v>-1138.010616391473</v>
       </c>
       <c r="J9">
-        <v>-0.1649989689662389</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>-0.1810506775998101</v>
+      </c>
+      <c r="K9">
+        <v>0.6966080402010055</v>
+      </c>
+      <c r="L9">
+        <v>0.6891303039276758</v>
+      </c>
+      <c r="M9">
+        <v>0.7325640309900395</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <v>3</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G10">
-        <v>6285.591589482498</v>
+        <v>1592.652152069054</v>
       </c>
       <c r="H10">
-        <v>5147.580973091025</v>
+        <v>1329.866189055798</v>
       </c>
       <c r="I10">
-        <v>-1138.010616391473</v>
+        <v>-262.7859630132555</v>
       </c>
       <c r="J10">
-        <v>-0.1810506775998101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>-0.1649989689662389</v>
+      </c>
+      <c r="K10">
+        <v>0.1765075376884422</v>
+      </c>
+      <c r="L10">
+        <v>0.1780352938278989</v>
+      </c>
+      <c r="M10">
+        <v>0.1691614661408112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D11">
         <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G11">
         <v>2548.713461124355</v>
@@ -1822,89 +2200,116 @@
       <c r="J11">
         <v>-0.00222421536994241</v>
       </c>
-    </row>
-    <row r="12" spans="1:10">
+      <c r="K11">
+        <v>0.1706372264187481</v>
+      </c>
+      <c r="L11">
+        <v>0.1789737600560029</v>
+      </c>
+      <c r="M11">
+        <v>0.007793264106436546</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D12">
         <v>4</v>
       </c>
       <c r="E12" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G12">
-        <v>2369.348836164419</v>
+        <v>10018.38219735946</v>
       </c>
       <c r="H12">
-        <v>2211.284760095633</v>
+        <v>9454.706519928746</v>
       </c>
       <c r="I12">
-        <v>-158.0640760687866</v>
+        <v>-563.675677430716</v>
       </c>
       <c r="J12">
-        <v>-0.06671203229181986</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>-0.05626414188702878</v>
+      </c>
+      <c r="K12">
+        <v>0.6707340693395321</v>
+      </c>
+      <c r="L12">
+        <v>0.6654009897232557</v>
+      </c>
+      <c r="M12">
+        <v>0.7749092401995692</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D13">
         <v>4</v>
       </c>
       <c r="E13" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G13">
-        <v>10018.38219735946</v>
+        <v>2369.348836164419</v>
       </c>
       <c r="H13">
-        <v>9454.706519928746</v>
+        <v>2211.284760095633</v>
       </c>
       <c r="I13">
-        <v>-563.675677430716</v>
+        <v>-158.0640760687866</v>
       </c>
       <c r="J13">
-        <v>-0.05626414188702878</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
+        <v>-0.06671203229181986</v>
+      </c>
+      <c r="K13">
+        <v>0.1586287042417198</v>
+      </c>
+      <c r="L13">
+        <v>0.1556252502207414</v>
+      </c>
+      <c r="M13">
+        <v>0.2172974956939943</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G14">
         <v>2443.987754662811</v>
@@ -1918,89 +2323,116 @@
       <c r="J14">
         <v>-0.01431517488000416</v>
       </c>
-    </row>
-    <row r="15" spans="1:10">
+      <c r="K14">
+        <v>0.4082140634723086</v>
+      </c>
+      <c r="L14">
+        <v>0.4104836703607108</v>
+      </c>
+      <c r="M14">
+        <v>0.2956548262474083</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D15">
         <v>5</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F15" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G15">
-        <v>771.1973555109769</v>
+        <v>2771.839770532215</v>
       </c>
       <c r="H15">
-        <v>741.4044825486761</v>
+        <v>2718.284437995423</v>
       </c>
       <c r="I15">
-        <v>-29.79287296230075</v>
+        <v>-53.55533253679232</v>
       </c>
       <c r="J15">
-        <v>-0.03863196981862146</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+        <v>-0.01932122235424498</v>
+      </c>
+      <c r="K15">
+        <v>0.4629744866210333</v>
+      </c>
+      <c r="L15">
+        <v>0.4631841479408621</v>
+      </c>
+      <c r="M15">
+        <v>0.4525765104974608</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D16">
         <v>5</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G16">
-        <v>2771.839770532215</v>
+        <v>771.1973555109769</v>
       </c>
       <c r="H16">
-        <v>2718.284437995423</v>
+        <v>741.4044825486761</v>
       </c>
       <c r="I16">
-        <v>-53.55533253679232</v>
+        <v>-29.79287296230075</v>
       </c>
       <c r="J16">
-        <v>-0.01932122235424498</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>-0.03863196981862146</v>
+      </c>
+      <c r="K16">
+        <v>0.1288114499066581</v>
+      </c>
+      <c r="L16">
+        <v>0.126332181698427</v>
+      </c>
+      <c r="M16">
+        <v>0.2517686632551309</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D17">
         <v>6</v>
       </c>
       <c r="E17" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G17">
         <v>737.9275791029602</v>
@@ -2014,89 +2446,116 @@
       <c r="J17">
         <v>0.02527738081884549</v>
       </c>
-    </row>
-    <row r="18" spans="1:10">
+      <c r="K17">
+        <v>0.7150284321689699</v>
+      </c>
+      <c r="L17">
+        <v>0.7220370319238563</v>
+      </c>
+      <c r="M17">
+        <v>1.179358721779987</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D18">
         <v>6</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F18" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G18">
-        <v>76.96177205368217</v>
+        <v>217.1361542691039</v>
       </c>
       <c r="H18">
-        <v>75.15174688619692</v>
+        <v>216.1094207703017</v>
       </c>
       <c r="I18">
-        <v>-1.81002516748525</v>
+        <v>-1.026733498802173</v>
       </c>
       <c r="J18">
-        <v>-0.02351849651048479</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
+        <v>-0.004728523917438958</v>
+      </c>
+      <c r="K18">
+        <v>0.2103980503655553</v>
+      </c>
+      <c r="L18">
+        <v>0.2062424473192178</v>
+      </c>
+      <c r="M18">
+        <v>-0.06491691032528364</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D19">
         <v>6</v>
       </c>
       <c r="E19" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F19" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G19">
-        <v>217.1361542691039</v>
+        <v>76.96177205368217</v>
       </c>
       <c r="H19">
-        <v>216.1094207703017</v>
+        <v>75.15174688619692</v>
       </c>
       <c r="I19">
-        <v>-1.026733498802173</v>
+        <v>-1.81002516748525</v>
       </c>
       <c r="J19">
-        <v>-0.004728523917438958</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
+        <v>-0.02351849651048479</v>
+      </c>
+      <c r="K19">
+        <v>0.07457351746547462</v>
+      </c>
+      <c r="L19">
+        <v>0.07172052075692592</v>
+      </c>
+      <c r="M19">
+        <v>-0.1144418114547037</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D20">
         <v>7</v>
       </c>
       <c r="E20" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F20" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G20">
         <v>28420.73848797222</v>
@@ -2110,89 +2569,116 @@
       <c r="J20">
         <v>0.03719956910429145</v>
       </c>
-    </row>
-    <row r="21" spans="1:10">
+      <c r="K20">
+        <v>0.1642038946162641</v>
+      </c>
+      <c r="L20">
+        <v>0.1684715681373224</v>
+      </c>
+      <c r="M20">
+        <v>0.5590864708306066</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D21">
         <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F21" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G21">
-        <v>19251.15945017174</v>
+        <v>125410.102061856</v>
       </c>
       <c r="H21">
-        <v>18859.45959321535</v>
+        <v>126635.5746934341</v>
       </c>
       <c r="I21">
-        <v>-391.6998569563912</v>
+        <v>1225.472631578057</v>
       </c>
       <c r="J21">
-        <v>-0.02034681900434297</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
+        <v>0.009771721826473095</v>
+      </c>
+      <c r="K21">
+        <v>0.7245704467353974</v>
+      </c>
+      <c r="L21">
+        <v>0.7237434690410091</v>
+      </c>
+      <c r="M21">
+        <v>0.6480512189124487</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D22">
         <v>7</v>
       </c>
       <c r="E22" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F22" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G22">
-        <v>125410.102061856</v>
+        <v>19251.15945017174</v>
       </c>
       <c r="H22">
-        <v>126635.5746934341</v>
+        <v>18859.45959321535</v>
       </c>
       <c r="I22">
-        <v>1225.472631578057</v>
+        <v>-391.6998569563912</v>
       </c>
       <c r="J22">
-        <v>0.009771721826473095</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
+        <v>-0.02034681900434297</v>
+      </c>
+      <c r="K22">
+        <v>0.1112256586483386</v>
+      </c>
+      <c r="L22">
+        <v>0.1077849628216685</v>
+      </c>
+      <c r="M22">
+        <v>-0.2071376897430553</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D23">
         <v>8</v>
       </c>
       <c r="E23" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F23" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G23">
         <v>19646.96893063571</v>
@@ -2206,89 +2692,116 @@
       <c r="J23">
         <v>0.05442807630137755</v>
       </c>
-    </row>
-    <row r="24" spans="1:10">
+      <c r="K23">
+        <v>0.1703395953757214</v>
+      </c>
+      <c r="L23">
+        <v>0.1771289185151771</v>
+      </c>
+      <c r="M23">
+        <v>0.6616646788393241</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>8</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F24" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G24">
-        <v>60774.34609826608</v>
+        <v>34918.68497109821</v>
       </c>
       <c r="H24">
-        <v>60014.07059865597</v>
+        <v>36225.75974666086</v>
       </c>
       <c r="I24">
-        <v>-760.2754996101139</v>
+        <v>1307.074775562643</v>
       </c>
       <c r="J24">
-        <v>-0.01250980962231702</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
+        <v>0.03743195875344372</v>
+      </c>
+      <c r="K24">
+        <v>0.3027456647398839</v>
+      </c>
+      <c r="L24">
+        <v>0.3097379743229643</v>
+      </c>
+      <c r="M24">
+        <v>0.8087603320261118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D25">
         <v>8</v>
       </c>
       <c r="E25" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F25" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G25">
-        <v>34918.68497109821</v>
+        <v>60774.34609826608</v>
       </c>
       <c r="H25">
-        <v>36225.75974666086</v>
+        <v>60014.07059865597</v>
       </c>
       <c r="I25">
-        <v>1307.074775562643</v>
+        <v>-760.2754996101139</v>
       </c>
       <c r="J25">
-        <v>0.03743195875344372</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10">
+        <v>-0.01250980962231702</v>
+      </c>
+      <c r="K25">
+        <v>0.5269147398843946</v>
+      </c>
+      <c r="L25">
+        <v>0.5131331071618586</v>
+      </c>
+      <c r="M25">
+        <v>-0.4704250108654359</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D26">
         <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F26" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G26">
         <v>6147.44206383908</v>
@@ -2302,89 +2815,116 @@
       <c r="J26">
         <v>0.02481979087750858</v>
       </c>
-    </row>
-    <row r="27" spans="1:10">
+      <c r="K26">
+        <v>0.08832531700918218</v>
+      </c>
+      <c r="L26">
+        <v>0.08787128903718494</v>
+      </c>
+      <c r="M26">
+        <v>0.07279481644886465</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D27">
         <v>9</v>
       </c>
       <c r="E27" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G27">
-        <v>34734.06209007435</v>
+        <v>28718.49584608657</v>
       </c>
       <c r="H27">
-        <v>35597.97077432211</v>
+        <v>29798.01293538272</v>
       </c>
       <c r="I27">
-        <v>863.9086842477554</v>
+        <v>1079.517089296154</v>
       </c>
       <c r="J27">
-        <v>0.02487208901761672</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10">
+        <v>0.03758961106743543</v>
+      </c>
+      <c r="K27">
+        <v>0.4126220667541173</v>
+      </c>
+      <c r="L27">
+        <v>0.415616091175496</v>
+      </c>
+      <c r="M27">
+        <v>0.5150357963516083</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D28">
         <v>9</v>
       </c>
       <c r="E28" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F28" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G28">
-        <v>28718.49584608657</v>
+        <v>34734.06209007435</v>
       </c>
       <c r="H28">
-        <v>29798.01293538272</v>
+        <v>35597.97077432211</v>
       </c>
       <c r="I28">
-        <v>1079.517089296154</v>
+        <v>863.9086842477554</v>
       </c>
       <c r="J28">
-        <v>0.03758961106743543</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10">
+        <v>0.02487208901761672</v>
+      </c>
+      <c r="K28">
+        <v>0.4990526162367004</v>
+      </c>
+      <c r="L28">
+        <v>0.4965126197873192</v>
+      </c>
+      <c r="M28">
+        <v>0.412169387199527</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D29">
         <v>10</v>
       </c>
       <c r="E29" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F29" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G29">
         <v>3914.073253833027</v>
@@ -2398,69 +2938,96 @@
       <c r="J29">
         <v>-0.07983986820489161</v>
       </c>
-    </row>
-    <row r="30" spans="1:10">
+      <c r="K29">
+        <v>0.08347529812606426</v>
+      </c>
+      <c r="L29">
+        <v>0.08631932144470537</v>
+      </c>
+      <c r="M29">
+        <v>0.06050142033165726</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D30">
         <v>10</v>
       </c>
       <c r="E30" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F30" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G30">
-        <v>10643.88287904598</v>
+        <v>32331.043867121</v>
       </c>
       <c r="H30">
-        <v>9488.084725005965</v>
+        <v>28634.18811389134</v>
       </c>
       <c r="I30">
-        <v>-1155.798154040016</v>
+        <v>-3696.855753229658</v>
       </c>
       <c r="J30">
-        <v>-0.1085880187873329</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
+        <v>-0.1143438414306557</v>
+      </c>
+      <c r="K30">
+        <v>0.6895229982964234</v>
+      </c>
+      <c r="L30">
+        <v>0.6862787152366686</v>
+      </c>
+      <c r="M30">
+        <v>0.7157301542141465</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D31">
         <v>10</v>
       </c>
       <c r="E31" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F31" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G31">
-        <v>32331.043867121</v>
+        <v>10643.88287904598</v>
       </c>
       <c r="H31">
-        <v>28634.18811389134</v>
+        <v>9488.084725005965</v>
       </c>
       <c r="I31">
-        <v>-3696.855753229658</v>
+        <v>-1155.798154040016</v>
       </c>
       <c r="J31">
-        <v>-0.1143438414306557</v>
+        <v>-0.1085880187873329</v>
+      </c>
+      <c r="K31">
+        <v>0.2270017035775125</v>
+      </c>
+      <c r="L31">
+        <v>0.227401963318626</v>
+      </c>
+      <c r="M31">
+        <v>0.2237684254541961</v>
       </c>
     </row>
   </sheetData>
@@ -2470,10 +3037,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2504,89 +3071,116 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G2">
-        <v>358.2232023220635</v>
+        <v>3451.96904055808</v>
       </c>
       <c r="H2">
-        <v>335.0327142331417</v>
+        <v>3302.062605575837</v>
       </c>
       <c r="I2">
-        <v>-23.19048808892177</v>
+        <v>-149.9064349822438</v>
       </c>
       <c r="J2">
-        <v>-0.06473753776583173</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>-0.04342635557299448</v>
+      </c>
+      <c r="K2">
+        <v>0.1624634248293149</v>
+      </c>
+      <c r="L2">
+        <v>0.1680227242756014</v>
+      </c>
+      <c r="M2">
+        <v>0.09397388447319024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G3">
-        <v>3451.96904055808</v>
+        <v>358.2232023220635</v>
       </c>
       <c r="H3">
-        <v>3302.062605575837</v>
+        <v>335.0327142331417</v>
       </c>
       <c r="I3">
-        <v>-149.9064349822438</v>
+        <v>-23.19048808892177</v>
       </c>
       <c r="J3">
-        <v>-0.04342635557299448</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>-0.06473753776583173</v>
+      </c>
+      <c r="K3">
+        <v>0.01685941201058921</v>
+      </c>
+      <c r="L3">
+        <v>0.01704786253048183</v>
+      </c>
+      <c r="M3">
+        <v>0.01453773648078125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G4">
         <v>12813.14065826372</v>
@@ -2600,25 +3194,34 @@
       <c r="J4">
         <v>-0.08095433323636185</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
+      <c r="K4">
+        <v>0.6030374808415785</v>
+      </c>
+      <c r="L4">
+        <v>0.5992049665301145</v>
+      </c>
+      <c r="M4">
+        <v>0.6502533479011925</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G5">
         <v>4624.335884521229</v>
@@ -2632,89 +3235,116 @@
       <c r="J5">
         <v>-0.08321547572827036</v>
       </c>
-    </row>
-    <row r="6" spans="1:10">
+      <c r="K5">
+        <v>0.2176396823185174</v>
+      </c>
+      <c r="L5">
+        <v>0.2157244466638025</v>
+      </c>
+      <c r="M5">
+        <v>0.241235031144836</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G6">
-        <v>109.9026098247154</v>
+        <v>1664.428681321303</v>
       </c>
       <c r="H6">
-        <v>105.7805933466526</v>
+        <v>1677.026407533276</v>
       </c>
       <c r="I6">
-        <v>-4.122016478062832</v>
+        <v>12.5977262119734</v>
       </c>
       <c r="J6">
-        <v>-0.03750608365567543</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>0.00756879904398951</v>
+      </c>
+      <c r="K6">
+        <v>0.2665394402035619</v>
+      </c>
+      <c r="L6">
+        <v>0.2745862662578333</v>
+      </c>
+      <c r="M6">
+        <v>-0.09187346646117013</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G7">
-        <v>1664.428681321303</v>
+        <v>109.9026098247154</v>
       </c>
       <c r="H7">
-        <v>1677.026407533276</v>
+        <v>105.7805933466526</v>
       </c>
       <c r="I7">
-        <v>12.5977262119734</v>
+        <v>-4.122016478062832</v>
       </c>
       <c r="J7">
-        <v>0.00756879904398951</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>-0.03750608365567543</v>
+      </c>
+      <c r="K7">
+        <v>0.01759966072943158</v>
+      </c>
+      <c r="L7">
+        <v>0.01731988121303284</v>
+      </c>
+      <c r="M7">
+        <v>0.03006129330622859</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D8">
         <v>2</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G8">
         <v>3583.089905851598</v>
@@ -2728,25 +3358,34 @@
       <c r="J8">
         <v>-0.03151553353281562</v>
       </c>
-    </row>
-    <row r="9" spans="1:10">
+      <c r="K8">
+        <v>0.5737913486005096</v>
+      </c>
+      <c r="L8">
+        <v>0.5681843603733253</v>
+      </c>
+      <c r="M8">
+        <v>0.8235316728707623</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D9">
         <v>2</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G9">
         <v>887.16564557301</v>
@@ -2760,89 +3399,116 @@
       <c r="J9">
         <v>-0.03682865426945892</v>
       </c>
-    </row>
-    <row r="10" spans="1:10">
+      <c r="K9">
+        <v>0.1420695504664969</v>
+      </c>
+      <c r="L9">
+        <v>0.1399094921558085</v>
+      </c>
+      <c r="M9">
+        <v>0.2382805002841791</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D10">
         <v>3</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G10">
-        <v>68.01361503497709</v>
+        <v>1144.895853088782</v>
       </c>
       <c r="H10">
-        <v>55.77432205469776</v>
+        <v>992.2301162322491</v>
       </c>
       <c r="I10">
-        <v>-12.23929298027934</v>
+        <v>-152.6657368565326</v>
       </c>
       <c r="J10">
-        <v>-0.1799535721485336</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>-0.1333446500349006</v>
+      </c>
+      <c r="K10">
+        <v>0.1268844221105523</v>
+      </c>
+      <c r="L10">
+        <v>0.1328344022444252</v>
+      </c>
+      <c r="M10">
+        <v>0.09827450286914927</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D11">
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G11">
-        <v>1144.895853088782</v>
+        <v>68.01361503497709</v>
       </c>
       <c r="H11">
-        <v>992.2301162322491</v>
+        <v>55.77432205469776</v>
       </c>
       <c r="I11">
-        <v>-152.6657368565326</v>
+        <v>-12.23929298027934</v>
       </c>
       <c r="J11">
-        <v>-0.1333446500349006</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
+        <v>-0.1799535721485336</v>
+      </c>
+      <c r="K11">
+        <v>0.007537688442211023</v>
+      </c>
+      <c r="L11">
+        <v>0.007466764623973264</v>
+      </c>
+      <c r="M11">
+        <v>0.007878718944232782</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D12">
         <v>3</v>
       </c>
       <c r="E12" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F12" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G12">
         <v>6183.571166930033</v>
@@ -2856,25 +3522,34 @@
       <c r="J12">
         <v>-0.1813075822358861</v>
       </c>
-    </row>
-    <row r="13" spans="1:10">
+      <c r="K12">
+        <v>0.685301507537689</v>
+      </c>
+      <c r="L12">
+        <v>0.6777324696106505</v>
+      </c>
+      <c r="M12">
+        <v>0.7216965137318911</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D13">
         <v>3</v>
       </c>
       <c r="E13" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G13">
         <v>1626.658959586543</v>
@@ -2888,89 +3563,116 @@
       <c r="J13">
         <v>-0.1644038210890883</v>
       </c>
-    </row>
-    <row r="14" spans="1:10">
+      <c r="K13">
+        <v>0.1802763819095477</v>
+      </c>
+      <c r="L13">
+        <v>0.181966363520951</v>
+      </c>
+      <c r="M13">
+        <v>0.1721502644547268</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D14">
         <v>4</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G14">
-        <v>257.4750261521749</v>
+        <v>2548.713461124355</v>
       </c>
       <c r="H14">
-        <v>251.5820998087408</v>
+        <v>2543.044573470543</v>
       </c>
       <c r="I14">
-        <v>-5.892926343434084</v>
+        <v>-5.668887653811908</v>
       </c>
       <c r="J14">
-        <v>-0.02288737059861954</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
+        <v>-0.00222421536994241</v>
+      </c>
+      <c r="K14">
+        <v>0.1706372264187481</v>
+      </c>
+      <c r="L14">
+        <v>0.1789737600560029</v>
+      </c>
+      <c r="M14">
+        <v>0.00779326410643653</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D15">
         <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G15">
-        <v>2548.713461124355</v>
+        <v>257.4750261521749</v>
       </c>
       <c r="H15">
-        <v>2543.044573470543</v>
+        <v>251.5820998087408</v>
       </c>
       <c r="I15">
-        <v>-5.668887653811908</v>
+        <v>-5.892926343434084</v>
       </c>
       <c r="J15">
-        <v>-0.00222421536994241</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+        <v>-0.02288737059861954</v>
+      </c>
+      <c r="K15">
+        <v>0.01723803989928318</v>
+      </c>
+      <c r="L15">
+        <v>0.01770578260219257</v>
+      </c>
+      <c r="M15">
+        <v>0.008101259745953486</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D16">
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G16">
         <v>9677.010814371186</v>
@@ -2984,25 +3686,34 @@
       <c r="J16">
         <v>-0.05677590087411744</v>
       </c>
-    </row>
-    <row r="17" spans="1:10">
+      <c r="K16">
+        <v>0.6478791400348646</v>
+      </c>
+      <c r="L16">
+        <v>0.6423792509026304</v>
+      </c>
+      <c r="M16">
+        <v>0.7553127302466282</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D17">
         <v>4</v>
       </c>
       <c r="E17" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F17" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G17">
         <v>2453.245193000522</v>
@@ -3016,89 +3727,116 @@
       <c r="J17">
         <v>-0.06783904881436519</v>
       </c>
-    </row>
-    <row r="18" spans="1:10">
+      <c r="K17">
+        <v>0.1642455936471043</v>
+      </c>
+      <c r="L17">
+        <v>0.1609412064391741</v>
+      </c>
+      <c r="M17">
+        <v>0.2287927459009819</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D18">
         <v>5</v>
       </c>
       <c r="E18" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G18">
-        <v>197.4563277395255</v>
+        <v>2443.987754662811</v>
       </c>
       <c r="H18">
-        <v>186.0946485799231</v>
+        <v>2409.001642550224</v>
       </c>
       <c r="I18">
-        <v>-11.36167915960237</v>
+        <v>-34.98611211258685</v>
       </c>
       <c r="J18">
-        <v>-0.05754021301657211</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
+        <v>-0.01431517488000416</v>
+      </c>
+      <c r="K18">
+        <v>0.4082140634723086</v>
+      </c>
+      <c r="L18">
+        <v>0.4104836703607108</v>
+      </c>
+      <c r="M18">
+        <v>0.2956548262474084</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D19">
         <v>5</v>
       </c>
       <c r="E19" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F19" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G19">
-        <v>2443.987754662811</v>
+        <v>197.4563277395255</v>
       </c>
       <c r="H19">
-        <v>2409.001642550224</v>
+        <v>186.0946485799231</v>
       </c>
       <c r="I19">
-        <v>-34.98611211258685</v>
+        <v>-11.36167915960237</v>
       </c>
       <c r="J19">
-        <v>-0.01431517488000416</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
+        <v>-0.05754021301657211</v>
+      </c>
+      <c r="K19">
+        <v>0.03298070939639072</v>
+      </c>
+      <c r="L19">
+        <v>0.03170973943492481</v>
+      </c>
+      <c r="M19">
+        <v>0.0960133914566213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D20">
         <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F20" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G20">
         <v>2563.206669524415</v>
@@ -3112,25 +3850,34 @@
       <c r="J20">
         <v>-0.01574273645324365</v>
       </c>
-    </row>
-    <row r="21" spans="1:10">
+      <c r="K20">
+        <v>0.4281269446172998</v>
+      </c>
+      <c r="L20">
+        <v>0.4298837628816293</v>
+      </c>
+      <c r="M20">
+        <v>0.3409990262160133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D21">
         <v>5</v>
       </c>
       <c r="E21" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F21" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G21">
         <v>782.3741287792515</v>
@@ -3144,89 +3891,116 @@
       <c r="J21">
         <v>-0.04043415816334739</v>
       </c>
-    </row>
-    <row r="22" spans="1:10">
+      <c r="K21">
+        <v>0.1306782825140009</v>
+      </c>
+      <c r="L21">
+        <v>0.1279228273227351</v>
+      </c>
+      <c r="M21">
+        <v>0.267332756079957</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
       <c r="A22" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D22">
         <v>6</v>
       </c>
       <c r="E22" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G22">
-        <v>75.03353593469043</v>
+        <v>737.9275791029602</v>
       </c>
       <c r="H22">
-        <v>75.0420923253308</v>
+        <v>756.5804555366744</v>
       </c>
       <c r="I22">
-        <v>0.008556390640364953</v>
+        <v>18.65287643371425</v>
       </c>
       <c r="J22">
-        <v>0.0001140342186167593</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
+        <v>0.02527738081884549</v>
+      </c>
+      <c r="K22">
+        <v>0.7150284321689699</v>
+      </c>
+      <c r="L22">
+        <v>0.7220370319238563</v>
+      </c>
+      <c r="M22">
+        <v>1.179358721779986</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D23">
         <v>6</v>
       </c>
       <c r="E23" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F23" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G23">
-        <v>737.9275791029602</v>
+        <v>75.03353593469043</v>
       </c>
       <c r="H23">
-        <v>756.5804555366744</v>
+        <v>75.0420923253308</v>
       </c>
       <c r="I23">
-        <v>18.65287643371425</v>
+        <v>0.008556390640364953</v>
       </c>
       <c r="J23">
-        <v>0.02527738081884549</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10">
+        <v>0.0001140342186167593</v>
+      </c>
+      <c r="K23">
+        <v>0.072705117790414</v>
+      </c>
+      <c r="L23">
+        <v>0.07161587272764458</v>
+      </c>
+      <c r="M23">
+        <v>0.0005409918392228188</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
       <c r="A24" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>6</v>
       </c>
       <c r="E24" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F24" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G24">
         <v>137.9108006844309</v>
@@ -3240,25 +4014,34 @@
       <c r="J24">
         <v>-0.008805413455624241</v>
       </c>
-    </row>
-    <row r="25" spans="1:10">
+      <c r="K24">
+        <v>0.133631194151096</v>
+      </c>
+      <c r="L24">
+        <v>0.1304552482347877</v>
+      </c>
+      <c r="M24">
+        <v>-0.0767800061860672</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D25">
         <v>6</v>
       </c>
       <c r="E25" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F25" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G25">
         <v>81.15358970366472</v>
@@ -3272,89 +4055,116 @@
       <c r="J25">
         <v>-0.02009712007639661</v>
       </c>
-    </row>
-    <row r="26" spans="1:10">
+      <c r="K25">
+        <v>0.07863525588951994</v>
+      </c>
+      <c r="L25">
+        <v>0.07589184711371147</v>
+      </c>
+      <c r="M25">
+        <v>-0.1031197074331419</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D26">
         <v>7</v>
       </c>
       <c r="E26" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F26" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G26">
-        <v>2795.482474226756</v>
+        <v>28420.73848797222</v>
       </c>
       <c r="H26">
-        <v>2720.328558298284</v>
+        <v>29477.97771335054</v>
       </c>
       <c r="I26">
-        <v>-75.15391592847118</v>
+        <v>1057.239225378318</v>
       </c>
       <c r="J26">
-        <v>-0.02688405905648152</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10">
+        <v>0.03719956910429145</v>
+      </c>
+      <c r="K26">
+        <v>0.1642038946162641</v>
+      </c>
+      <c r="L26">
+        <v>0.1684715681373224</v>
+      </c>
+      <c r="M26">
+        <v>0.5590864708306125</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D27">
         <v>7</v>
       </c>
       <c r="E27" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F27" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G27">
-        <v>28420.73848797222</v>
+        <v>2795.482474226756</v>
       </c>
       <c r="H27">
-        <v>29477.97771335054</v>
+        <v>2720.328558298284</v>
       </c>
       <c r="I27">
-        <v>1057.239225378318</v>
+        <v>-75.15391592847118</v>
       </c>
       <c r="J27">
-        <v>0.03719956910429145</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10">
+        <v>-0.02688405905648152</v>
+      </c>
+      <c r="K27">
+        <v>0.01615120274914061</v>
+      </c>
+      <c r="L27">
+        <v>0.01554713225316305</v>
+      </c>
+      <c r="M27">
+        <v>-0.03974269646542306</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D28">
         <v>7</v>
       </c>
       <c r="E28" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F28" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G28">
         <v>122029.7491408939</v>
@@ -3368,25 +4178,34 @@
       <c r="J28">
         <v>0.01052237457105928</v>
       </c>
-    </row>
-    <row r="29" spans="1:10">
+      <c r="K28">
+        <v>0.7050400916380323</v>
+      </c>
+      <c r="L28">
+        <v>0.7047589251659383</v>
+      </c>
+      <c r="M28">
+        <v>0.6790241041690427</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B29" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D29">
         <v>7</v>
       </c>
       <c r="E29" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F29" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G29">
         <v>19836.02989690712</v>
@@ -3400,89 +4219,116 @@
       <c r="J29">
         <v>-0.01891084257648035</v>
       </c>
-    </row>
-    <row r="30" spans="1:10">
+      <c r="K29">
+        <v>0.114604810996563</v>
+      </c>
+      <c r="L29">
+        <v>0.1112223744435762</v>
+      </c>
+      <c r="M29">
+        <v>-0.1983678785342321</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
       <c r="A30" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D30">
         <v>8</v>
       </c>
       <c r="E30" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F30" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G30">
-        <v>822.964234104015</v>
+        <v>19646.96893063571</v>
       </c>
       <c r="H30">
-        <v>879.2572806078971</v>
+        <v>20716.31565468315</v>
       </c>
       <c r="I30">
-        <v>56.29304650388212</v>
+        <v>1069.346724047435</v>
       </c>
       <c r="J30">
-        <v>0.06840278613707922</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
+        <v>0.05442807630137755</v>
+      </c>
+      <c r="K30">
+        <v>0.1703395953757214</v>
+      </c>
+      <c r="L30">
+        <v>0.1771289185151771</v>
+      </c>
+      <c r="M30">
+        <v>0.6616646788393236</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B31" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D31">
         <v>8</v>
       </c>
       <c r="E31" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F31" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G31">
-        <v>19646.96893063571</v>
+        <v>822.964234104015</v>
       </c>
       <c r="H31">
-        <v>20716.31565468315</v>
+        <v>879.2572806078971</v>
       </c>
       <c r="I31">
-        <v>1069.346724047435</v>
+        <v>56.29304650388212</v>
       </c>
       <c r="J31">
-        <v>0.05442807630137755</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10">
+        <v>0.06840278613707922</v>
+      </c>
+      <c r="K31">
+        <v>0.007135115606936144</v>
+      </c>
+      <c r="L31">
+        <v>0.007517837332019279</v>
+      </c>
+      <c r="M31">
+        <v>0.03483165908518372</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B32" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D32">
         <v>8</v>
       </c>
       <c r="E32" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F32" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G32">
         <v>29126.68352601153</v>
@@ -3496,25 +4342,34 @@
       <c r="J32">
         <v>0.03735969350004975</v>
       </c>
-    </row>
-    <row r="33" spans="1:10">
+      <c r="K32">
+        <v>0.2525289017341038</v>
+      </c>
+      <c r="L32">
+        <v>0.2583433921909181</v>
+      </c>
+      <c r="M32">
+        <v>0.6733079617836275</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
       <c r="A33" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B33" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D33">
         <v>8</v>
       </c>
       <c r="E33" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F33" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G33">
         <v>65743.38330924875</v>
@@ -3528,89 +4383,116 @@
       <c r="J33">
         <v>-0.009090766396137271</v>
       </c>
-    </row>
-    <row r="34" spans="1:10">
+      <c r="K33">
+        <v>0.5699963872832385</v>
+      </c>
+      <c r="L33">
+        <v>0.5570098519618856</v>
+      </c>
+      <c r="M33">
+        <v>-0.3698042997081348</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B34" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D34">
         <v>9</v>
       </c>
       <c r="E34" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F34" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G34">
-        <v>50.72146917358625</v>
+        <v>6147.44206383908</v>
       </c>
       <c r="H34">
-        <v>51.50919573397206</v>
+        <v>6300.020290295166</v>
       </c>
       <c r="I34">
-        <v>0.7877265603858064</v>
+        <v>152.5782264560858</v>
       </c>
       <c r="J34">
-        <v>0.01553043658277989</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10">
+        <v>0.02481979087750858</v>
+      </c>
+      <c r="K34">
+        <v>0.08832531700918218</v>
+      </c>
+      <c r="L34">
+        <v>0.08787128903718494</v>
+      </c>
+      <c r="M34">
+        <v>0.07279481644886471</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B35" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D35">
         <v>9</v>
       </c>
       <c r="E35" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F35" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G35">
-        <v>6147.44206383908</v>
+        <v>50.72146917358625</v>
       </c>
       <c r="H35">
-        <v>6300.020290295166</v>
+        <v>51.50919573397206</v>
       </c>
       <c r="I35">
-        <v>152.5782264560858</v>
+        <v>0.7877265603858064</v>
       </c>
       <c r="J35">
-        <v>0.02481979087750858</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10">
+        <v>0.01553043658277989</v>
+      </c>
+      <c r="K35">
+        <v>0.0007287567409998024</v>
+      </c>
+      <c r="L35">
+        <v>0.0007184388649327244</v>
+      </c>
+      <c r="M35">
+        <v>0.000375823023422574</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
       <c r="A36" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B36" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C36" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D36">
         <v>9</v>
       </c>
       <c r="E36" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F36" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G36">
         <v>12365.89418452115</v>
@@ -3624,25 +4506,34 @@
       <c r="J36">
         <v>0.02147291423728611</v>
       </c>
-    </row>
-    <row r="37" spans="1:10">
+      <c r="K36">
+        <v>0.1776708934557636</v>
+      </c>
+      <c r="L36">
+        <v>0.1761803345387664</v>
+      </c>
+      <c r="M36">
+        <v>0.126684770301764</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
       <c r="A37" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C37" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D37">
         <v>9</v>
       </c>
       <c r="E37" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F37" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G37">
         <v>51035.94228246618</v>
@@ -3656,89 +4547,116 @@
       <c r="J37">
         <v>0.03286127749752801</v>
       </c>
-    </row>
-    <row r="38" spans="1:10">
+      <c r="K37">
+        <v>0.7332750327940544</v>
+      </c>
+      <c r="L37">
+        <v>0.735229937559116</v>
+      </c>
+      <c r="M37">
+        <v>0.8001445902259487</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B38" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C38" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D38">
         <v>10</v>
       </c>
       <c r="E38" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F38" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G38">
-        <v>129.8034497444613</v>
+        <v>3914.073253833027</v>
       </c>
       <c r="H38">
-        <v>104.1471664191177</v>
+        <v>3601.574161102707</v>
       </c>
       <c r="I38">
-        <v>-25.65628332534352</v>
+        <v>-312.4990927303202</v>
       </c>
       <c r="J38">
-        <v>-0.1976548649196304</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10">
+        <v>-0.07983986820489161</v>
+      </c>
+      <c r="K38">
+        <v>0.08347529812606425</v>
+      </c>
+      <c r="L38">
+        <v>0.08631932144470537</v>
+      </c>
+      <c r="M38">
+        <v>0.06050142033165718</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
       <c r="A39" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B39" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D39">
         <v>10</v>
       </c>
       <c r="E39" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F39" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G39">
-        <v>3914.073253833027</v>
+        <v>129.8034497444613</v>
       </c>
       <c r="H39">
-        <v>3601.574161102707</v>
+        <v>104.1471664191177</v>
       </c>
       <c r="I39">
-        <v>-312.4990927303202</v>
+        <v>-25.65628332534352</v>
       </c>
       <c r="J39">
-        <v>-0.07983986820489161</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10">
+        <v>-0.1976548649196304</v>
+      </c>
+      <c r="K39">
+        <v>0.002768313458262305</v>
+      </c>
+      <c r="L39">
+        <v>0.002496106517194297</v>
+      </c>
+      <c r="M39">
+        <v>0.004967187482218536</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B40" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C40" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D40">
         <v>10</v>
       </c>
       <c r="E40" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F40" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G40">
         <v>5821.185477001693</v>
@@ -3752,25 +4670,34 @@
       <c r="J40">
         <v>-0.1302839422527272</v>
       </c>
-    </row>
-    <row r="41" spans="1:10">
+      <c r="K40">
+        <v>0.1241482112436113</v>
+      </c>
+      <c r="L40">
+        <v>0.1213401651212456</v>
+      </c>
+      <c r="M40">
+        <v>0.1468314670500763</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B41" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C41" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D41">
         <v>10</v>
       </c>
       <c r="E41" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F41" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G41">
         <v>37023.93781942083</v>
@@ -3783,6 +4710,15 @@
       </c>
       <c r="J41">
         <v>-0.1098908131074611</v>
+      </c>
+      <c r="K41">
+        <v>0.7896081771720621</v>
+      </c>
+      <c r="L41">
+        <v>0.7898444069168546</v>
+      </c>
+      <c r="M41">
+        <v>0.787699925136048</v>
       </c>
     </row>
   </sheetData>

</xml_diff>